<commit_message>
IPO Desk: accuracy pass - Maxwell revenue base corrected (Rs 29.45 cr ops, fair value Rs 49/84/122), BLS band confirmed by NSE
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Sh3XfYSpHMqTXgPXQV3Xds
</commit_message>
<xml_diff>
--- a/ipo-analysis/companies/maxwell-engineering-solutions-ltd/MAXWELL_ENGINEERING_SOLU_01_Screening.xlsx
+++ b/ipo-analysis/companies/maxwell-engineering-solutions-ltd/MAXWELL_ENGINEERING_SOLU_01_Screening.xlsx
@@ -1311,14 +1311,14 @@
         <v>22.59</v>
       </c>
       <c r="E5" s="16" t="n">
-        <v>30.76</v>
+        <v>29.45</v>
       </c>
       <c r="F5" s="16" t="n">
         <v>12.25</v>
       </c>
       <c r="G5" s="7" t="inlineStr">
         <is>
-          <t>Restated total income FY24-26 and 4M to Jul-2026 (HDFC Sky, Chittorgarh, unp.me)</t>
+          <t>Restated total income FY24-26 and 4M to Jul-2026 (HDFC Sky, Chittorgarh, unp.me); FY26 revenue from operations Rs 29.45 cr (total income Rs 30.76 cr less other income Rs 1.31 cr), corrected 29-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -1330,7 +1330,9 @@
       </c>
       <c r="C6" s="16" t="n"/>
       <c r="D6" s="16" t="n"/>
-      <c r="E6" s="16" t="n"/>
+      <c r="E6" s="16" t="n">
+        <v>1.31</v>
+      </c>
       <c r="F6" s="16" t="n"/>
       <c r="G6" s="7" t="inlineStr"/>
     </row>

</xml_diff>